<commit_message>
#167 Top Board Client BOM missing Part no Added
</commit_message>
<xml_diff>
--- a/Design-Files/LSS_Top_Board_v3.4/BOM/Client_BOM-LSS_Top_Board_v3.4.xlsx
+++ b/Design-Files/LSS_Top_Board_v3.4/BOM/Client_BOM-LSS_Top_Board_v3.4.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LiberDB\Documents\GitHub\ColeBenson-SmartMotors\Design-Files\LSS_Top_Board_v3.4\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\ColeBenson-SmartMotors\Design-Files\LSS_Top_Board_v3.4\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="512" uniqueCount="374">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="525" uniqueCount="381">
   <si>
     <t>Description</t>
   </si>
@@ -1150,6 +1150,27 @@
   </si>
   <si>
     <t># Symbol is used for 220nF in PCB</t>
+  </si>
+  <si>
+    <t>ISO6762FQDWRQ1</t>
+  </si>
+  <si>
+    <t>ISO7740FDBQR</t>
+  </si>
+  <si>
+    <t>MSMP12A-M3/89A</t>
+  </si>
+  <si>
+    <t>MSP3V3HM3/89A</t>
+  </si>
+  <si>
+    <t>Vishay Intertech</t>
+  </si>
+  <si>
+    <t>USBLC6-4SC6</t>
+  </si>
+  <si>
+    <t>USBLC6-2P6</t>
   </si>
 </sst>
 </file>
@@ -2201,8 +2222,12 @@
       <c r="C25" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="D25" s="1"/>
-      <c r="E25" s="1"/>
+      <c r="D25" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>127</v>
+      </c>
       <c r="F25" s="2" t="s">
         <v>365</v>
       </c>
@@ -2221,8 +2246,12 @@
       <c r="C26" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="D26" s="1"/>
-      <c r="E26" s="1"/>
+      <c r="D26" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>127</v>
+      </c>
       <c r="F26" s="2" t="s">
         <v>365</v>
       </c>
@@ -2313,8 +2342,12 @@
       <c r="C30" s="5" t="s">
         <v>138</v>
       </c>
-      <c r="D30" s="1"/>
-      <c r="E30" s="1"/>
+      <c r="D30" s="2" t="s">
+        <v>376</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>378</v>
+      </c>
       <c r="F30" s="2" t="s">
         <v>365</v>
       </c>
@@ -2333,8 +2366,12 @@
       <c r="C31" s="5" t="s">
         <v>138</v>
       </c>
-      <c r="D31" s="1"/>
-      <c r="E31" s="1"/>
+      <c r="D31" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>378</v>
+      </c>
       <c r="F31" s="2" t="s">
         <v>365</v>
       </c>
@@ -2374,7 +2411,9 @@
       <c r="B33" s="6" t="s">
         <v>145</v>
       </c>
-      <c r="C33" s="6"/>
+      <c r="C33" s="6" t="s">
+        <v>368</v>
+      </c>
       <c r="D33" s="6" t="s">
         <v>361</v>
       </c>
@@ -3481,8 +3520,12 @@
       <c r="C79" s="5" t="s">
         <v>333</v>
       </c>
-      <c r="D79" s="1"/>
-      <c r="E79" s="1"/>
+      <c r="D79" s="2" t="s">
+        <v>379</v>
+      </c>
+      <c r="E79" s="1" t="s">
+        <v>151</v>
+      </c>
       <c r="F79" s="2" t="s">
         <v>365</v>
       </c>
@@ -3501,8 +3544,12 @@
       <c r="C80" s="5" t="s">
         <v>334</v>
       </c>
-      <c r="D80" s="1"/>
-      <c r="E80" s="1"/>
+      <c r="D80" s="2" t="s">
+        <v>380</v>
+      </c>
+      <c r="E80" s="1" t="s">
+        <v>151</v>
+      </c>
       <c r="F80" s="2" t="s">
         <v>365</v>
       </c>

</xml_diff>

<commit_message>
#174 C22 Update in Client BOM.
</commit_message>
<xml_diff>
--- a/Design-Files/LSS_Top_Board_v3.4/BOM/Client_BOM-LSS_Top_Board_v3.4.xlsx
+++ b/Design-Files/LSS_Top_Board_v3.4/BOM/Client_BOM-LSS_Top_Board_v3.4.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="525" uniqueCount="381">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="526" uniqueCount="381">
   <si>
     <t>Description</t>
   </si>
@@ -212,16 +212,7 @@
     <t>220uF</t>
   </si>
   <si>
-    <t>220uF ±20% 63V 10mm 14.5mm 1.2A 100kHz 10000hrs 105℃ -55℃~+105℃ SMD,10x14.5mm Aluminum Electrolytic Capacitors - SMD RoHS</t>
-  </si>
-  <si>
     <t>C22</t>
-  </si>
-  <si>
-    <t>VKME1451J221MV</t>
-  </si>
-  <si>
-    <t>Ymin</t>
   </si>
   <si>
     <t>1000pF</t>
@@ -1171,6 +1162,15 @@
   </si>
   <si>
     <t>USBLC6-2P6</t>
+  </si>
+  <si>
+    <t>220uF 63V 225mA@100KHz ±20% SMD,D10xL10.5mm Aluminum Electrolytic Capacitors - SMD ROHS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KNSCHA </t>
+  </si>
+  <si>
+    <t>189RV0038</t>
   </si>
 </sst>
 </file>
@@ -1648,16 +1648,16 @@
         <v>3</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="G1" s="21" t="s">
         <v>4</v>
       </c>
       <c r="H1" s="23" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="I1" s="21" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="30" x14ac:dyDescent="0.25">
@@ -1684,7 +1684,7 @@
       </c>
       <c r="H2" s="24"/>
       <c r="I2" s="27" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="60" x14ac:dyDescent="0.25">
@@ -1903,18 +1903,21 @@
       </c>
       <c r="H11" s="24"/>
     </row>
-    <row r="12" spans="1:9" ht="150" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" ht="120" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>61</v>
+        <v>378</v>
+      </c>
+      <c r="C12" s="10" t="s">
+        <v>365</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>63</v>
+        <v>380</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>64</v>
+        <v>379</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>60</v>
@@ -1926,22 +1929,22 @@
     </row>
     <row r="13" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="12" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="C13" s="5" t="s">
         <v>9</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="G13" s="20">
         <v>1</v>
@@ -1950,22 +1953,22 @@
     </row>
     <row r="14" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A14" s="12" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C14" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="E14" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="D14" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>73</v>
-      </c>
       <c r="F14" s="2" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="G14" s="20">
         <v>1</v>
@@ -1974,22 +1977,22 @@
     </row>
     <row r="15" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A15" s="12" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="C15" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="E15" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="D15" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>77</v>
-      </c>
       <c r="F15" s="2" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="G15" s="20">
         <v>1</v>
@@ -1998,22 +2001,22 @@
     </row>
     <row r="16" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A16" s="12" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="C16" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="D16" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="D16" s="2" t="s">
-        <v>81</v>
-      </c>
       <c r="E16" s="2" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="G16" s="20">
         <v>2</v>
@@ -2022,22 +2025,22 @@
     </row>
     <row r="17" spans="1:8" ht="165" x14ac:dyDescent="0.25">
       <c r="A17" s="12" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C17" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="E17" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="D17" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>85</v>
-      </c>
       <c r="F17" s="2" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="G17" s="20">
         <v>4</v>
@@ -2046,22 +2049,22 @@
     </row>
     <row r="18" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="12" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B18" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E18" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="C18" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>90</v>
-      </c>
       <c r="F18" s="2" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="G18" s="20">
         <v>1</v>
@@ -2070,22 +2073,22 @@
     </row>
     <row r="19" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A19" s="12" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="C19" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="E19" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="D19" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>94</v>
-      </c>
       <c r="F19" s="2" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="G19" s="20">
         <v>1</v>
@@ -2094,22 +2097,22 @@
     </row>
     <row r="20" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A20" s="12" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="G20" s="20">
         <v>1</v>
@@ -2118,22 +2121,22 @@
     </row>
     <row r="21" spans="1:8" ht="120" x14ac:dyDescent="0.25">
       <c r="A21" s="12" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="B21" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="E21" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="C21" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="E21" s="2" t="s">
-        <v>102</v>
-      </c>
       <c r="F21" s="2" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="G21" s="20">
         <v>1</v>
@@ -2142,22 +2145,22 @@
     </row>
     <row r="22" spans="1:8" ht="75" x14ac:dyDescent="0.25">
       <c r="A22" s="12" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B22" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="E22" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="C22" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="E22" s="2" t="s">
-        <v>107</v>
-      </c>
       <c r="F22" s="2" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="G22" s="20">
         <v>1</v>
@@ -2166,22 +2169,22 @@
     </row>
     <row r="23" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="12" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="C23" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="E23" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="D23" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>111</v>
-      </c>
       <c r="F23" s="2" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="G23" s="20">
         <v>8</v>
@@ -2190,22 +2193,22 @@
     </row>
     <row r="24" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A24" s="12" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="B24" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="E24" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="C24" s="5" t="s">
-        <v>115</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="E24" s="2" t="s">
-        <v>116</v>
-      </c>
       <c r="F24" s="2" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="G24" s="20">
         <v>1</v>
@@ -2214,22 +2217,22 @@
     </row>
     <row r="25" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A25" s="12" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="G25" s="20">
         <v>1</v>
@@ -2238,22 +2241,22 @@
     </row>
     <row r="26" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A26" s="12" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="G26" s="20">
         <v>1</v>
@@ -2262,22 +2265,22 @@
     </row>
     <row r="27" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A27" s="12" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="C27" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="E27" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="D27" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="E27" s="2" t="s">
-        <v>127</v>
-      </c>
       <c r="F27" s="2" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="G27" s="20">
         <v>1</v>
@@ -2286,22 +2289,22 @@
     </row>
     <row r="28" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A28" s="12" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="C28" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="E28" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="D28" s="2" t="s">
-        <v>128</v>
-      </c>
-      <c r="E28" s="2" t="s">
-        <v>131</v>
-      </c>
       <c r="F28" s="2" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="G28" s="20">
         <v>1</v>
@@ -2310,22 +2313,22 @@
     </row>
     <row r="29" spans="1:8" ht="90" x14ac:dyDescent="0.25">
       <c r="A29" s="12" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="C29" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="E29" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="D29" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="E29" s="2" t="s">
-        <v>135</v>
-      </c>
       <c r="F29" s="2" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="G29" s="20">
         <v>1</v>
@@ -2334,22 +2337,22 @@
     </row>
     <row r="30" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A30" s="12" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="G30" s="20">
         <v>1</v>
@@ -2358,22 +2361,22 @@
     </row>
     <row r="31" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A31" s="12" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="G31" s="20">
         <v>2</v>
@@ -2382,22 +2385,22 @@
     </row>
     <row r="32" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A32" s="12" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="D32" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="E32" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="E32" s="2" t="s">
-        <v>144</v>
-      </c>
       <c r="F32" s="2" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="G32" s="20">
         <v>2</v>
@@ -2406,49 +2409,49 @@
     </row>
     <row r="33" spans="1:9" s="8" customFormat="1" ht="60" x14ac:dyDescent="0.25">
       <c r="A33" s="7" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="E33" s="7" t="s">
+        <v>359</v>
+      </c>
+      <c r="F33" s="6" t="s">
         <v>362</v>
-      </c>
-      <c r="F33" s="6" t="s">
-        <v>365</v>
       </c>
       <c r="G33" s="20">
         <v>2</v>
       </c>
       <c r="H33" s="25" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="I33" s="20"/>
     </row>
     <row r="34" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A34" s="12" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="B34" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="E34" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="C34" s="5" t="s">
-        <v>150</v>
-      </c>
-      <c r="D34" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="E34" s="2" t="s">
-        <v>151</v>
-      </c>
       <c r="F34" s="2" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="G34" s="20">
         <v>1</v>
@@ -2457,18 +2460,18 @@
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="12" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="D35" s="1"/>
       <c r="E35" s="1"/>
       <c r="F35" s="2" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="G35" s="20">
         <v>4</v>
@@ -2477,22 +2480,22 @@
     </row>
     <row r="36" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A36" s="12" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="B36" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="C36" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="E36" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="C36" s="5" t="s">
-        <v>158</v>
-      </c>
-      <c r="D36" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="E36" s="2" t="s">
-        <v>159</v>
-      </c>
       <c r="F36" s="2" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="G36" s="20">
         <v>1</v>
@@ -2501,22 +2504,22 @@
     </row>
     <row r="37" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A37" s="12" t="s">
+        <v>159</v>
+      </c>
+      <c r="B37" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="C37" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="D37" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="B37" s="5" t="s">
+      <c r="E37" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="C37" s="5" t="s">
-        <v>163</v>
-      </c>
-      <c r="D37" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="E37" s="2" t="s">
-        <v>164</v>
-      </c>
       <c r="F37" s="2" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="G37" s="20">
         <v>1</v>
@@ -2525,22 +2528,22 @@
     </row>
     <row r="38" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A38" s="12" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="B38" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="C38" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="D38" s="2" t="s">
         <v>167</v>
-      </c>
-      <c r="C38" s="5" t="s">
-        <v>169</v>
-      </c>
-      <c r="D38" s="2" t="s">
-        <v>170</v>
       </c>
       <c r="E38" s="2" t="s">
         <v>48</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="G38" s="20">
         <v>1</v>
@@ -2549,22 +2552,22 @@
     </row>
     <row r="39" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A39" s="12" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="C39" s="5" t="s">
         <v>9</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="G39" s="20">
         <v>1</v>
@@ -2573,22 +2576,22 @@
     </row>
     <row r="40" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A40" s="12" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="C40" s="5" t="s">
         <v>9</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="G40" s="20">
         <v>2</v>
@@ -2597,22 +2600,22 @@
     </row>
     <row r="41" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A41" s="12" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="C41" s="5" t="s">
         <v>26</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="G41" s="20">
         <v>2</v>
@@ -2621,22 +2624,22 @@
     </row>
     <row r="42" spans="1:9" ht="60" x14ac:dyDescent="0.25">
       <c r="A42" s="12" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="C42" s="5" t="s">
         <v>20</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="E42" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="G42" s="20">
         <v>12</v>
@@ -2645,22 +2648,22 @@
     </row>
     <row r="43" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A43" s="12" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="C43" s="5" t="s">
         <v>20</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="F43" s="2" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="G43" s="20">
         <v>1</v>
@@ -2669,22 +2672,22 @@
     </row>
     <row r="44" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A44" s="12" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="C44" s="5" t="s">
         <v>20</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="E44" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="G44" s="20">
         <v>4</v>
@@ -2693,22 +2696,22 @@
     </row>
     <row r="45" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A45" s="12" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="C45" s="5" t="s">
         <v>20</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="G45" s="20">
         <v>1</v>
@@ -2717,22 +2720,22 @@
     </row>
     <row r="46" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A46" s="12" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="C46" s="5" t="s">
         <v>26</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="G46" s="20">
         <v>2</v>
@@ -2741,22 +2744,22 @@
     </row>
     <row r="47" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A47" s="12" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="C47" s="5" t="s">
         <v>26</v>
       </c>
       <c r="D47" s="2" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="F47" s="2" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="G47" s="20">
         <v>1</v>
@@ -2765,22 +2768,22 @@
     </row>
     <row r="48" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A48" s="12" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="B48" s="5" t="s">
+        <v>206</v>
+      </c>
+      <c r="C48" s="5" t="s">
+        <v>208</v>
+      </c>
+      <c r="D48" s="2" t="s">
         <v>209</v>
       </c>
-      <c r="C48" s="5" t="s">
-        <v>211</v>
-      </c>
-      <c r="D48" s="2" t="s">
-        <v>212</v>
-      </c>
       <c r="E48" s="2" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="F48" s="2" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="G48" s="20">
         <v>2</v>
@@ -2789,22 +2792,22 @@
     </row>
     <row r="49" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A49" s="12" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="C49" s="5" t="s">
         <v>20</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="F49" s="2" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="G49" s="20">
         <v>1</v>
@@ -2813,22 +2816,22 @@
     </row>
     <row r="50" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A50" s="12" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="C50" s="5" t="s">
         <v>20</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="E50" s="2" t="s">
         <v>48</v>
       </c>
       <c r="F50" s="2" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="G50" s="20">
         <v>6</v>
@@ -2837,22 +2840,22 @@
     </row>
     <row r="51" spans="1:8" ht="75" x14ac:dyDescent="0.25">
       <c r="A51" s="12" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C51" s="5" t="s">
         <v>26</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="F51" s="2" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="G51" s="20">
         <v>1</v>
@@ -2861,22 +2864,22 @@
     </row>
     <row r="52" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A52" s="12" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="C52" s="5" t="s">
         <v>20</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="E52" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F52" s="2" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="G52" s="20">
         <v>1</v>
@@ -2885,22 +2888,22 @@
     </row>
     <row r="53" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A53" s="12" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="B53" s="5" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="C53" s="5" t="s">
         <v>26</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="F53" s="2" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="G53" s="20">
         <v>2</v>
@@ -2909,22 +2912,22 @@
     </row>
     <row r="54" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A54" s="12" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="C54" s="5" t="s">
         <v>26</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="F54" s="2" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="G54" s="20">
         <v>6</v>
@@ -2933,22 +2936,22 @@
     </row>
     <row r="55" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A55" s="12" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="B55" s="5" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="C55" s="5" t="s">
         <v>20</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="E55" s="2" t="s">
         <v>48</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="G55" s="20">
         <v>7</v>
@@ -2957,22 +2960,22 @@
     </row>
     <row r="56" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A56" s="12" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="B56" s="5" t="s">
+        <v>235</v>
+      </c>
+      <c r="C56" s="5" t="s">
+        <v>208</v>
+      </c>
+      <c r="D56" s="2" t="s">
         <v>238</v>
       </c>
-      <c r="C56" s="5" t="s">
-        <v>211</v>
-      </c>
-      <c r="D56" s="2" t="s">
-        <v>241</v>
-      </c>
       <c r="E56" s="2" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="F56" s="2" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="G56" s="20">
         <v>1</v>
@@ -2981,22 +2984,22 @@
     </row>
     <row r="57" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A57" s="12" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="B57" s="5" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="C57" s="5" t="s">
         <v>20</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="F57" s="2" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="G57" s="20">
         <v>1</v>
@@ -3005,22 +3008,22 @@
     </row>
     <row r="58" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A58" s="12" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="B58" s="5" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="C58" s="5" t="s">
         <v>26</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="F58" s="2" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="G58" s="20">
         <v>4</v>
@@ -3029,22 +3032,22 @@
     </row>
     <row r="59" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A59" s="12" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="C59" s="5" t="s">
         <v>26</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="F59" s="2" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="G59" s="20">
         <v>2</v>
@@ -3053,22 +3056,22 @@
     </row>
     <row r="60" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A60" s="12" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="B60" s="5" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="C60" s="5" t="s">
         <v>26</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="F60" s="2" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="G60" s="20">
         <v>1</v>
@@ -3077,22 +3080,22 @@
     </row>
     <row r="61" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A61" s="12" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="B61" s="5" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="C61" s="5" t="s">
         <v>20</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="F61" s="2" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="G61" s="20">
         <v>1</v>
@@ -3101,22 +3104,22 @@
     </row>
     <row r="62" spans="1:8" ht="90" x14ac:dyDescent="0.25">
       <c r="A62" s="12" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="B62" s="5" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="C62" s="5" t="s">
         <v>26</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="F62" s="2" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="G62" s="20">
         <v>2</v>
@@ -3125,22 +3128,22 @@
     </row>
     <row r="63" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A63" s="12" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="B63" s="5" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="C63" s="5" t="s">
         <v>26</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="E63" s="2" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="F63" s="2" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="G63" s="20">
         <v>1</v>
@@ -3149,22 +3152,22 @@
     </row>
     <row r="64" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A64" s="12" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="B64" s="5" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="C64" s="5" t="s">
         <v>26</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="E64" s="2" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="F64" s="2" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="G64" s="20">
         <v>1</v>
@@ -3173,22 +3176,22 @@
     </row>
     <row r="65" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A65" s="12" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="B65" s="5" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="C65" s="5" t="s">
         <v>26</v>
       </c>
       <c r="D65" s="2" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="E65" s="2" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="F65" s="2" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="G65" s="20">
         <v>2</v>
@@ -3197,22 +3200,22 @@
     </row>
     <row r="66" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A66" s="12" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="B66" s="5" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="C66" s="5" t="s">
         <v>26</v>
       </c>
       <c r="D66" s="2" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="E66" s="2" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="F66" s="2" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="G66" s="20">
         <v>1</v>
@@ -3221,22 +3224,22 @@
     </row>
     <row r="67" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A67" s="12" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="B67" s="5" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="C67" s="5" t="s">
         <v>20</v>
       </c>
       <c r="D67" s="2" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="E67" s="2" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="F67" s="2" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="G67" s="20">
         <v>1</v>
@@ -3245,22 +3248,22 @@
     </row>
     <row r="68" spans="1:9" ht="105" x14ac:dyDescent="0.25">
       <c r="A68" s="12" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="B68" s="5" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="C68" s="5" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="D68" s="2" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="E68" s="2" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="F68" s="2" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="G68" s="20">
         <v>4</v>
@@ -3269,49 +3272,49 @@
     </row>
     <row r="69" spans="1:9" ht="105" x14ac:dyDescent="0.25">
       <c r="A69" s="12" t="s">
+        <v>288</v>
+      </c>
+      <c r="B69" s="5" t="s">
+        <v>287</v>
+      </c>
+      <c r="C69" s="5" t="s">
+        <v>289</v>
+      </c>
+      <c r="D69" s="2" t="s">
         <v>291</v>
       </c>
-      <c r="B69" s="5" t="s">
+      <c r="E69" s="2" t="s">
         <v>290</v>
       </c>
-      <c r="C69" s="5" t="s">
-        <v>292</v>
-      </c>
-      <c r="D69" s="2" t="s">
-        <v>294</v>
-      </c>
-      <c r="E69" s="2" t="s">
-        <v>293</v>
-      </c>
       <c r="F69" s="2" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="G69" s="20">
         <v>8</v>
       </c>
       <c r="H69" s="24"/>
       <c r="I69" s="27" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
     </row>
     <row r="70" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A70" s="12" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="B70" s="5" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="C70" s="5" t="s">
+        <v>292</v>
+      </c>
+      <c r="D70" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="E70" s="2" t="s">
         <v>295</v>
       </c>
-      <c r="D70" s="2" t="s">
-        <v>295</v>
-      </c>
-      <c r="E70" s="2" t="s">
-        <v>298</v>
-      </c>
       <c r="F70" s="2" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="G70" s="20">
         <v>1</v>
@@ -3320,22 +3323,22 @@
     </row>
     <row r="71" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A71" s="12" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="B71" s="5" t="s">
+        <v>297</v>
+      </c>
+      <c r="C71" s="5" t="s">
+        <v>299</v>
+      </c>
+      <c r="D71" s="2" t="s">
         <v>300</v>
       </c>
-      <c r="C71" s="5" t="s">
-        <v>302</v>
-      </c>
-      <c r="D71" s="2" t="s">
-        <v>303</v>
-      </c>
       <c r="E71" s="2" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="F71" s="2" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="G71" s="20">
         <v>2</v>
@@ -3344,22 +3347,22 @@
     </row>
     <row r="72" spans="1:9" ht="105" x14ac:dyDescent="0.25">
       <c r="A72" s="12" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="B72" s="5" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="C72" s="5" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="D72" s="2" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="F72" s="2" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="G72" s="20">
         <v>1</v>
@@ -3368,22 +3371,22 @@
     </row>
     <row r="73" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A73" s="12" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="B73" s="5" t="s">
+        <v>306</v>
+      </c>
+      <c r="C73" s="5" t="s">
+        <v>308</v>
+      </c>
+      <c r="D73" s="2" t="s">
+        <v>305</v>
+      </c>
+      <c r="E73" s="2" t="s">
         <v>309</v>
       </c>
-      <c r="C73" s="5" t="s">
-        <v>311</v>
-      </c>
-      <c r="D73" s="2" t="s">
-        <v>308</v>
-      </c>
-      <c r="E73" s="2" t="s">
-        <v>312</v>
-      </c>
       <c r="F73" s="2" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="G73" s="20">
         <v>1</v>
@@ -3392,22 +3395,22 @@
     </row>
     <row r="74" spans="1:9" ht="105" x14ac:dyDescent="0.25">
       <c r="A74" s="12" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="B74" s="5" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="C74" s="5" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="E74" s="2" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="F74" s="2" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="G74" s="20">
         <v>1</v>
@@ -3416,22 +3419,22 @@
     </row>
     <row r="75" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="A75" s="12" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="B75" s="5" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="C75" s="5" t="s">
+        <v>314</v>
+      </c>
+      <c r="D75" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="E75" s="2" t="s">
         <v>317</v>
       </c>
-      <c r="D75" s="2" t="s">
-        <v>317</v>
-      </c>
-      <c r="E75" s="2" t="s">
-        <v>320</v>
-      </c>
       <c r="F75" s="2" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="G75" s="20">
         <v>1</v>
@@ -3440,19 +3443,19 @@
     </row>
     <row r="76" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A76" s="12" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="B76" s="5" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
       <c r="C76" s="5" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
       <c r="D76" s="2" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
       <c r="E76" s="2" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="F76" s="2" t="s">
         <v>60</v>
@@ -3464,22 +3467,22 @@
     </row>
     <row r="77" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A77" s="12" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="B77" s="5" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="C77" s="5" t="s">
+        <v>321</v>
+      </c>
+      <c r="D77" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="E77" s="2" t="s">
         <v>324</v>
       </c>
-      <c r="D77" s="2" t="s">
-        <v>324</v>
-      </c>
-      <c r="E77" s="2" t="s">
-        <v>327</v>
-      </c>
       <c r="F77" s="2" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="G77" s="20">
         <v>1</v>
@@ -3488,22 +3491,22 @@
     </row>
     <row r="78" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A78" s="12" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="B78" s="5" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="C78" s="5" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="D78" s="2" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="E78" s="2" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="F78" s="2" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="G78" s="20">
         <v>1</v>
@@ -3512,22 +3515,22 @@
     </row>
     <row r="79" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A79" s="12" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="B79" s="5" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="C79" s="5" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="D79" s="2" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
       <c r="E79" s="1" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="F79" s="2" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="G79" s="20">
         <v>1</v>
@@ -3536,22 +3539,22 @@
     </row>
     <row r="80" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A80" s="12" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="B80" s="5" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="C80" s="5" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
       <c r="E80" s="1" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="F80" s="2" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="G80" s="20">
         <v>2</v>
@@ -3560,22 +3563,22 @@
     </row>
     <row r="81" spans="1:18" ht="45" x14ac:dyDescent="0.25">
       <c r="A81" s="12" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="B81" s="5" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="C81" s="5" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="E81" s="2" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="F81" s="2" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="G81" s="20">
         <v>1</v>
@@ -3584,22 +3587,22 @@
     </row>
     <row r="82" spans="1:18" ht="105" x14ac:dyDescent="0.25">
       <c r="A82" s="12" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="B82" s="5" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="C82" s="5" t="s">
         <v>26</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
       <c r="E82" s="2" t="s">
         <v>31</v>
       </c>
       <c r="F82" s="2" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="G82" s="20">
         <v>1</v>
@@ -3608,22 +3611,22 @@
     </row>
     <row r="83" spans="1:18" ht="90" x14ac:dyDescent="0.25">
       <c r="A83" s="12" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="B83" s="5" t="s">
+        <v>342</v>
+      </c>
+      <c r="C83" s="5" t="s">
+        <v>341</v>
+      </c>
+      <c r="D83" s="2" t="s">
         <v>345</v>
       </c>
-      <c r="C83" s="5" t="s">
+      <c r="E83" s="2" t="s">
         <v>344</v>
       </c>
-      <c r="D83" s="2" t="s">
-        <v>348</v>
-      </c>
-      <c r="E83" s="2" t="s">
-        <v>347</v>
-      </c>
       <c r="F83" s="2" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="G83" s="20">
         <v>1</v>
@@ -3632,22 +3635,22 @@
     </row>
     <row r="84" spans="1:18" ht="105" x14ac:dyDescent="0.25">
       <c r="A84" s="12" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="B84" s="5" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="C84" s="5" t="s">
         <v>26</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="E84" s="2" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="F84" s="2" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="G84" s="20">
         <v>1</v>
@@ -3656,22 +3659,22 @@
     </row>
     <row r="85" spans="1:18" ht="75" x14ac:dyDescent="0.25">
       <c r="A85" s="12" t="s">
-        <v>356</v>
+        <v>353</v>
       </c>
       <c r="B85" s="5" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
       <c r="C85" s="5" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="D85" s="2" t="s">
+        <v>351</v>
+      </c>
+      <c r="E85" s="2" t="s">
         <v>354</v>
       </c>
-      <c r="E85" s="2" t="s">
-        <v>357</v>
-      </c>
       <c r="F85" s="2" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="G85" s="20">
         <v>2</v>
@@ -3680,22 +3683,22 @@
     </row>
     <row r="86" spans="1:18" ht="90" x14ac:dyDescent="0.25">
       <c r="A86" s="12" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
       <c r="B86" s="5" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
       <c r="C86" s="5" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
       <c r="E86" s="2" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
       <c r="F86" s="2" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="G86" s="20">
         <v>1</v>
@@ -3709,22 +3712,22 @@
     </row>
     <row r="87" spans="1:18" ht="30" x14ac:dyDescent="0.25">
       <c r="A87" s="12" t="s">
+        <v>363</v>
+      </c>
+      <c r="B87" s="5" t="s">
+        <v>364</v>
+      </c>
+      <c r="C87" s="5" t="s">
+        <v>365</v>
+      </c>
+      <c r="D87" s="5" t="s">
         <v>366</v>
       </c>
-      <c r="B87" s="5" t="s">
+      <c r="E87" s="5" t="s">
         <v>367</v>
       </c>
-      <c r="C87" s="5" t="s">
-        <v>368</v>
-      </c>
-      <c r="D87" s="5" t="s">
-        <v>369</v>
-      </c>
-      <c r="E87" s="5" t="s">
-        <v>370</v>
-      </c>
       <c r="F87" s="18" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="G87" s="20">
         <v>1</v>

</xml_diff>